<commit_message>
XGBoost feature engeneering script
</commit_message>
<xml_diff>
--- a/RandomForest_Outputs/agriculture_berries_best_random_forest_results.xlsx
+++ b/RandomForest_Outputs/agriculture_berries_best_random_forest_results.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/Python Projects/Parameter-Optimisation/RandomForest_Search_Outputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/Python Projects/Parameter-Optimisation/RandomForest_Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD3F05B7899E3D7F05015087657ABE163" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C3BF412-D4BF-4B77-A626-5CE58D283758}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_2B59D2BFD3F05B7899E3D7F05015087657ABE163" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B2DF2C9-E468-4638-878F-A3A607FE9054}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$10</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -410,6 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="16.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -460,7 +464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -507,7 +511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -554,7 +558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -601,7 +605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -648,7 +652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -695,7 +699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -789,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -836,7 +840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -884,6 +888,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="C1:C10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="8229714302"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>